<commit_message>
feat(xlsx-mmc): aggiungi group row NIOSH/Snook-Ciriello al template e aggiorna offset schema
- build-mmc-template.py: PAGE_ROWS 13→14, group row in r3 (B:I=NIOSH, J:M=Snook)
- mmc.xlsx: rigenerato con nuova struttura
- exportSchemas.ts: blocchi MMC aggiornati (dataStartRow +1, headerRow/footerRow per PAGE_ROWS=14)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/mmc.xlsx
+++ b/public/templates/mmc.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Foglio1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Foglio1'!$A$1:$N$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Foglio1'!$A$1:$N$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -96,6 +96,10 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -481,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -536,1120 +540,1184 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Sollevamento (NIOSH)</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Spinta·Traino·Trasporto (Snook-Ciriello)</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>REG
 [n°]</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>CARICO
 (kg)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>H. MANI
 (cm)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>DIST. VERT.
 (cm)</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>DIST. PESO/
 CORPO (cm)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>DISLOC.
 (°)</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>FREQ.
 GESTI</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>GIUDIZIO
 PRESA</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>N°
 PERS.</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>F. MANTEN.
 (kg)</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>SPINTA
 (kg)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>TRAINO
 (kg)</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>DIST. TRASP.
 (m)</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="6" t="n">
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="6" t="n">
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="9" t="n"/>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="9" t="n"/>
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="9" t="n"/>
+      <c r="N7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-    </row>
-    <row r="12" ht="27.75" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="27.75" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Tecnico rilevatore</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="C13" s="11" t="n"/>
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1"/>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="14" ht="15" customHeight="1"/>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Impresa:</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="B15" s="2" t="n"/>
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Data:</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Cantiere:</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n"/>
-      <c r="M14" s="1" t="inlineStr">
+      <c r="F15" s="2" t="n"/>
+      <c r="M15" s="1" t="inlineStr">
         <is>
           <t>Progressiva:</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>Pag: 2</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24.95" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16" ht="24.95" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>MONITORAGGIO MMC — MOVIMENTAZIONE MANUALE CARICHI (D.Lgs 81/08 — Titolo VI)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Sollevamento (NIOSH)</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>Spinta·Traino·Trasporto (Snook-Ciriello)</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="n"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>REG
 [n°]</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>CARICO
 (kg)</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>H. MANI
 (cm)</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>DIST. VERT.
 (cm)</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>DIST. PESO/
 CORPO (cm)</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>DISLOC.
 (°)</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>FREQ.
 GESTI</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>GIUDIZIO
 PRESA</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>N°
 PERS.</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>F. MANTEN.
 (kg)</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>SPINTA
 (kg)</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>TRAINO
 (kg)</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
         <is>
           <t>DIST. TRASP.
 (m)</t>
         </is>
       </c>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="N18" s="7" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="6" t="n">
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="6" t="n">
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="9" t="n"/>
+      <c r="L19" s="9" t="n"/>
+      <c r="M19" s="9" t="n"/>
+      <c r="N19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="6" t="n">
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="n"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" s="9" t="n"/>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="9" t="n"/>
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="9" t="n"/>
+      <c r="N20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="6" t="n">
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
+      <c r="I21" s="9" t="n"/>
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="9" t="n"/>
+      <c r="L21" s="9" t="n"/>
+      <c r="M21" s="9" t="n"/>
+      <c r="N21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="6" t="n">
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="6" t="n">
+      <c r="B23" s="9" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9" t="n"/>
+      <c r="N23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-    </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="6" t="n">
+      <c r="B24" s="9" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="9" t="n"/>
+      <c r="L24" s="9" t="n"/>
+      <c r="M24" s="9" t="n"/>
+      <c r="N24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
-      <c r="N23" s="7" t="n"/>
-    </row>
-    <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="6" t="n">
+      <c r="B25" s="9" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n"/>
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="9" t="n"/>
+      <c r="L25" s="9" t="n"/>
+      <c r="M25" s="9" t="n"/>
+      <c r="N25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
-      <c r="N24" s="7" t="n"/>
-    </row>
-    <row r="25" ht="27.75" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="9" t="n"/>
+      <c r="N26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="27.75" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Tecnico rilevatore</t>
         </is>
       </c>
-      <c r="C25" s="9" t="n"/>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="C27" s="11" t="n"/>
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>Impresa:</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="B29" s="2" t="n"/>
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Data:</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Cantiere:</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n"/>
-      <c r="M27" s="1" t="inlineStr">
+      <c r="F29" s="2" t="n"/>
+      <c r="M29" s="1" t="inlineStr">
         <is>
           <t>Progressiva:</t>
         </is>
       </c>
-      <c r="N27" s="3" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>Pag: 3</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24.95" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="30" ht="24.95" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>MONITORAGGIO MMC — MOVIMENTAZIONE MANUALE CARICHI (D.Lgs 81/08 — Titolo VI)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Sollevamento (NIOSH)</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>Spinta·Traino·Trasporto (Snook-Ciriello)</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>REG
 [n°]</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>CARICO
 (kg)</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>H. MANI
 (cm)</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>DIST. VERT.
 (cm)</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>DIST. PESO/
 CORPO (cm)</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>DISLOC.
 (°)</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>FREQ.
 GESTI</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>GIUDIZIO
 PRESA</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>N°
 PERS.</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>F. MANTEN.
 (kg)</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>SPINTA
 (kg)</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="L32" s="7" t="inlineStr">
         <is>
           <t>TRAINO
 (kg)</t>
         </is>
       </c>
-      <c r="M29" s="5" t="inlineStr">
+      <c r="M32" s="7" t="inlineStr">
         <is>
           <t>DIST. TRASP.
 (m)</t>
         </is>
       </c>
-      <c r="N29" s="5" t="inlineStr">
+      <c r="N32" s="7" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="6" t="n">
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
-      <c r="I30" s="7" t="n"/>
-      <c r="J30" s="7" t="n"/>
-      <c r="K30" s="7" t="n"/>
-      <c r="L30" s="7" t="n"/>
-      <c r="M30" s="7" t="n"/>
-      <c r="N30" s="7" t="n"/>
-    </row>
-    <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="6" t="n">
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="9" t="n"/>
+      <c r="L33" s="9" t="n"/>
+      <c r="M33" s="9" t="n"/>
+      <c r="N33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
-      <c r="F31" s="7" t="n"/>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="7" t="n"/>
-      <c r="N31" s="7" t="n"/>
-    </row>
-    <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="6" t="n">
+      <c r="B34" s="9" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
+      <c r="K34" s="9" t="n"/>
+      <c r="L34" s="9" t="n"/>
+      <c r="M34" s="9" t="n"/>
+      <c r="N34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
-      <c r="F32" s="7" t="n"/>
-      <c r="G32" s="7" t="n"/>
-      <c r="H32" s="7" t="n"/>
-      <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
-      <c r="L32" s="7" t="n"/>
-      <c r="M32" s="7" t="n"/>
-      <c r="N32" s="7" t="n"/>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="6" t="n">
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="9" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="6" t="n">
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="9" t="n"/>
+      <c r="L36" s="9" t="n"/>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="7" t="n"/>
-      <c r="I34" s="7" t="n"/>
-      <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
-      <c r="M34" s="7" t="n"/>
-      <c r="N34" s="7" t="n"/>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="6" t="n">
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="9" t="n"/>
+      <c r="M37" s="9" t="n"/>
+      <c r="N37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
-      <c r="N35" s="7" t="n"/>
-    </row>
-    <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="6" t="n">
+      <c r="B38" s="9" t="n"/>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="9" t="n"/>
+      <c r="F38" s="9" t="n"/>
+      <c r="G38" s="9" t="n"/>
+      <c r="H38" s="9" t="n"/>
+      <c r="I38" s="9" t="n"/>
+      <c r="J38" s="9" t="n"/>
+      <c r="K38" s="9" t="n"/>
+      <c r="L38" s="9" t="n"/>
+      <c r="M38" s="9" t="n"/>
+      <c r="N38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="7" t="n"/>
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
-      <c r="M36" s="7" t="n"/>
-      <c r="N36" s="7" t="n"/>
-    </row>
-    <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="6" t="n">
+      <c r="B39" s="9" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="9" t="n"/>
+      <c r="L39" s="9" t="n"/>
+      <c r="M39" s="9" t="n"/>
+      <c r="N39" s="9" t="n"/>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
-      <c r="F37" s="7" t="n"/>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
-      <c r="M37" s="7" t="n"/>
-      <c r="N37" s="7" t="n"/>
-    </row>
-    <row r="38" ht="27.75" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="B40" s="9" t="n"/>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
+      <c r="J40" s="9" t="n"/>
+      <c r="K40" s="9" t="n"/>
+      <c r="L40" s="9" t="n"/>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="9" t="n"/>
+    </row>
+    <row r="41" ht="27.75" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Tecnico rilevatore</t>
         </is>
       </c>
-      <c r="C38" s="9" t="n"/>
-      <c r="F38" s="10" t="inlineStr">
+      <c r="C41" s="11" t="n"/>
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1"/>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="1" t="inlineStr">
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>Impresa:</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n"/>
-      <c r="D40" s="1" t="inlineStr">
+      <c r="B43" s="2" t="n"/>
+      <c r="D43" s="1" t="inlineStr">
         <is>
           <t>Data:</t>
         </is>
       </c>
-      <c r="E40" s="1" t="inlineStr">
+      <c r="E43" s="1" t="inlineStr">
         <is>
           <t>Cantiere:</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n"/>
-      <c r="M40" s="1" t="inlineStr">
+      <c r="F43" s="2" t="n"/>
+      <c r="M43" s="1" t="inlineStr">
         <is>
           <t>Progressiva:</t>
         </is>
       </c>
-      <c r="N40" s="3" t="inlineStr">
+      <c r="N43" s="3" t="inlineStr">
         <is>
           <t>Pag: 4</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="24.95" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="44" ht="24.95" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>MONITORAGGIO MMC — MOVIMENTAZIONE MANUALE CARICHI (D.Lgs 81/08 — Titolo VI)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Sollevamento (NIOSH)</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>Spinta·Traino·Trasporto (Snook-Ciriello)</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="n"/>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>REG
 [n°]</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>CARICO
 (kg)</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>H. MANI
 (cm)</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>DIST. VERT.
 (cm)</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>DIST. PESO/
 CORPO (cm)</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>DISLOC.
 (°)</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>FREQ.
 GESTI</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
+      <c r="H46" s="7" t="inlineStr">
         <is>
           <t>GIUDIZIO
 PRESA</t>
         </is>
       </c>
-      <c r="I42" s="5" t="inlineStr">
+      <c r="I46" s="7" t="inlineStr">
         <is>
           <t>N°
 PERS.</t>
         </is>
       </c>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="J46" s="7" t="inlineStr">
         <is>
           <t>F. MANTEN.
 (kg)</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr">
+      <c r="K46" s="7" t="inlineStr">
         <is>
           <t>SPINTA
 (kg)</t>
         </is>
       </c>
-      <c r="L42" s="5" t="inlineStr">
+      <c r="L46" s="7" t="inlineStr">
         <is>
           <t>TRAINO
 (kg)</t>
         </is>
       </c>
-      <c r="M42" s="5" t="inlineStr">
+      <c r="M46" s="7" t="inlineStr">
         <is>
           <t>DIST. TRASP.
 (m)</t>
         </is>
       </c>
-      <c r="N42" s="5" t="inlineStr">
+      <c r="N46" s="7" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="6" t="n">
+    <row r="47" ht="36" customHeight="1">
+      <c r="A47" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="B43" s="7" t="n"/>
-      <c r="C43" s="7" t="n"/>
-      <c r="D43" s="7" t="n"/>
-      <c r="E43" s="7" t="n"/>
-      <c r="F43" s="7" t="n"/>
-      <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="n"/>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="n"/>
-      <c r="M43" s="7" t="n"/>
-      <c r="N43" s="7" t="n"/>
-    </row>
-    <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="6" t="n">
+      <c r="B47" s="9" t="n"/>
+      <c r="C47" s="9" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="9" t="n"/>
+      <c r="I47" s="9" t="n"/>
+      <c r="J47" s="9" t="n"/>
+      <c r="K47" s="9" t="n"/>
+      <c r="L47" s="9" t="n"/>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="9" t="n"/>
+    </row>
+    <row r="48" ht="36" customHeight="1">
+      <c r="A48" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="B44" s="7" t="n"/>
-      <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
-      <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="n"/>
-      <c r="G44" s="7" t="n"/>
-      <c r="H44" s="7" t="n"/>
-      <c r="I44" s="7" t="n"/>
-      <c r="J44" s="7" t="n"/>
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
-      <c r="M44" s="7" t="n"/>
-      <c r="N44" s="7" t="n"/>
-    </row>
-    <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="6" t="n">
+      <c r="B48" s="9" t="n"/>
+      <c r="C48" s="9" t="n"/>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="9" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="9" t="n"/>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="9" t="n"/>
+    </row>
+    <row r="49" ht="36" customHeight="1">
+      <c r="A49" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="B45" s="7" t="n"/>
-      <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
-      <c r="E45" s="7" t="n"/>
-      <c r="F45" s="7" t="n"/>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="7" t="n"/>
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
-      <c r="M45" s="7" t="n"/>
-      <c r="N45" s="7" t="n"/>
-    </row>
-    <row r="46" ht="36" customHeight="1">
-      <c r="A46" s="6" t="n">
+      <c r="B49" s="9" t="n"/>
+      <c r="C49" s="9" t="n"/>
+      <c r="D49" s="9" t="n"/>
+      <c r="E49" s="9" t="n"/>
+      <c r="F49" s="9" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n"/>
+      <c r="I49" s="9" t="n"/>
+      <c r="J49" s="9" t="n"/>
+      <c r="K49" s="9" t="n"/>
+      <c r="L49" s="9" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="9" t="n"/>
+    </row>
+    <row r="50" ht="36" customHeight="1">
+      <c r="A50" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="7" t="n"/>
-      <c r="D46" s="7" t="n"/>
-      <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="n"/>
-      <c r="G46" s="7" t="n"/>
-      <c r="H46" s="7" t="n"/>
-      <c r="I46" s="7" t="n"/>
-      <c r="J46" s="7" t="n"/>
-      <c r="K46" s="7" t="n"/>
-      <c r="L46" s="7" t="n"/>
-      <c r="M46" s="7" t="n"/>
-      <c r="N46" s="7" t="n"/>
-    </row>
-    <row r="47" ht="36" customHeight="1">
-      <c r="A47" s="6" t="n">
+      <c r="B50" s="9" t="n"/>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n"/>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="9" t="n"/>
+      <c r="K50" s="9" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="36" customHeight="1">
+      <c r="A51" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B47" s="7" t="n"/>
-      <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
-      <c r="E47" s="7" t="n"/>
-      <c r="F47" s="7" t="n"/>
-      <c r="G47" s="7" t="n"/>
-      <c r="H47" s="7" t="n"/>
-      <c r="I47" s="7" t="n"/>
-      <c r="J47" s="7" t="n"/>
-      <c r="K47" s="7" t="n"/>
-      <c r="L47" s="7" t="n"/>
-      <c r="M47" s="7" t="n"/>
-      <c r="N47" s="7" t="n"/>
-    </row>
-    <row r="48" ht="36" customHeight="1">
-      <c r="A48" s="6" t="n">
+      <c r="B51" s="9" t="n"/>
+      <c r="C51" s="9" t="n"/>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="9" t="n"/>
+      <c r="F51" s="9" t="n"/>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" s="9" t="n"/>
+      <c r="J51" s="9" t="n"/>
+      <c r="K51" s="9" t="n"/>
+      <c r="L51" s="9" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="9" t="n"/>
+    </row>
+    <row r="52" ht="36" customHeight="1">
+      <c r="A52" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="7" t="n"/>
-      <c r="H48" s="7" t="n"/>
-      <c r="I48" s="7" t="n"/>
-      <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
-      <c r="L48" s="7" t="n"/>
-      <c r="M48" s="7" t="n"/>
-      <c r="N48" s="7" t="n"/>
-    </row>
-    <row r="49" ht="36" customHeight="1">
-      <c r="A49" s="6" t="n">
+      <c r="B52" s="9" t="n"/>
+      <c r="C52" s="9" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="9" t="n"/>
+      <c r="G52" s="9" t="n"/>
+      <c r="H52" s="9" t="n"/>
+      <c r="I52" s="9" t="n"/>
+      <c r="J52" s="9" t="n"/>
+      <c r="K52" s="9" t="n"/>
+      <c r="L52" s="9" t="n"/>
+      <c r="M52" s="9" t="n"/>
+      <c r="N52" s="9" t="n"/>
+    </row>
+    <row r="53" ht="36" customHeight="1">
+      <c r="A53" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="n"/>
-      <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="7" t="n"/>
-      <c r="H49" s="7" t="n"/>
-      <c r="I49" s="7" t="n"/>
-      <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
-      <c r="L49" s="7" t="n"/>
-      <c r="M49" s="7" t="n"/>
-      <c r="N49" s="7" t="n"/>
-    </row>
-    <row r="50" ht="36" customHeight="1">
-      <c r="A50" s="6" t="n">
+      <c r="B53" s="9" t="n"/>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="9" t="n"/>
+      <c r="J53" s="9" t="n"/>
+      <c r="K53" s="9" t="n"/>
+      <c r="L53" s="9" t="n"/>
+      <c r="M53" s="9" t="n"/>
+      <c r="N53" s="9" t="n"/>
+    </row>
+    <row r="54" ht="36" customHeight="1">
+      <c r="A54" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B50" s="7" t="n"/>
-      <c r="C50" s="7" t="n"/>
-      <c r="D50" s="7" t="n"/>
-      <c r="E50" s="7" t="n"/>
-      <c r="F50" s="7" t="n"/>
-      <c r="G50" s="7" t="n"/>
-      <c r="H50" s="7" t="n"/>
-      <c r="I50" s="7" t="n"/>
-      <c r="J50" s="7" t="n"/>
-      <c r="K50" s="7" t="n"/>
-      <c r="L50" s="7" t="n"/>
-      <c r="M50" s="7" t="n"/>
-      <c r="N50" s="7" t="n"/>
-    </row>
-    <row r="51" ht="27.75" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="B54" s="9" t="n"/>
+      <c r="C54" s="9" t="n"/>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="F54" s="9" t="n"/>
+      <c r="G54" s="9" t="n"/>
+      <c r="H54" s="9" t="n"/>
+      <c r="I54" s="9" t="n"/>
+      <c r="J54" s="9" t="n"/>
+      <c r="K54" s="9" t="n"/>
+      <c r="L54" s="9" t="n"/>
+      <c r="M54" s="9" t="n"/>
+      <c r="N54" s="9" t="n"/>
+    </row>
+    <row r="55" ht="27.75" customHeight="1">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>Tecnico rilevatore</t>
         </is>
       </c>
-      <c r="C51" s="9" t="n"/>
-      <c r="F51" s="10" t="inlineStr">
+      <c r="C55" s="11" t="n"/>
+      <c r="F55" s="12" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="F51:N51"/>
-    <mergeCell ref="F27:L27"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="F38:N38"/>
+  <mergeCells count="32">
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="J31:M31"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="A30:N30"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="F43:L43"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="F41:N41"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B43:C43"/>
     <mergeCell ref="F1:L1"/>
-    <mergeCell ref="F14:L14"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="A41:N41"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A16:N16"/>
+    <mergeCell ref="F29:L29"/>
+    <mergeCell ref="F13:N13"/>
+    <mergeCell ref="F27:N27"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="F40:L40"/>
+    <mergeCell ref="F55:N55"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="C13:E13"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="F25:N25"/>
-    <mergeCell ref="A28:N28"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="F12:N12"/>
+    <mergeCell ref="F15:L15"/>
+    <mergeCell ref="J45:M45"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="A44:N44"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="3" manualBreakCount="3">
-    <brk id="13" min="0" max="16383" man="1"/>
-    <brk id="26" min="0" max="16383" man="1"/>
-    <brk id="39" min="0" max="16383" man="1"/>
+    <brk id="14" min="0" max="16383" man="1"/>
+    <brk id="28" min="0" max="16383" man="1"/>
+    <brk id="42" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>